<commit_message>
Correct KSI-CMT-IMM to KSI-CMT-RMV per CR26; evaluate TLS minimum in control-plane assertion; rename Class C method count check
</commit_message>
<xml_diff>
--- a/03-northgate-signal-fedramp-20x/artifacts/ksi_validation_register.xlsx
+++ b/03-northgate-signal-fedramp-20x/artifacts/ksi_validation_register.xlsx
@@ -521,6 +521,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="11">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1020,7 +1021,7 @@
     <row r="12" ht="46.25" customHeight="1" s="11">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>KSI-CMT-IMM</t>
+          <t>KSI-CMT-RMV</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -1030,17 +1031,17 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Deploying Immutable Resources</t>
+          <t>Redeploying vs Modifying</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Changes are executed through redeployment of version controlled immutable resources rather than direct modification wherever possible.</t>
+          <t>Execute changes to machine-based information resources through redeployment of version controlled immutable resources rather than direct modification wherever reasonable.</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>CM-02, CM-03, CM-04, CM-08, SA-11</t>
+          <t>CM-02, CM-03, CM-05, CM-06, CM-07, CM-08(01), SI-03</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
@@ -1401,6 +1402,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1577,6 +1579,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -1766,6 +1769,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.85" customHeight="1" s="11">
       <c r="A3" s="17" t="inlineStr">
         <is>

</xml_diff>